<commit_message>
data(km19): sinh lại bộ file cắt thép sau khi sửa dầm Super-T theo bản vẽ
- Nguồn: BBS đã sửa (dầm 89,69 t thay vì 361,6 t). 0 lỗi đọc, 0 thanh chưa lập kế hoạch.
- 19.953 cây 11,7 m (bản trước 37.682), đề-xê chung 1,9%; Ø16 FEASIBLE (60 s/Ø), các Ø khác OPTIMAL.
- Nối chồng 40d đã gồm trong chiều dài BBS; tổng đoạn = chiều dài BBS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/00_BANG_TONG_HOP_CAT_THEP_THEO_PHI.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/00_BANG_TONG_HOP_CAT_THEP_THEO_PHI.xlsx
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>77681</v>
+        <v>21068</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>138949.04</v>
+        <v>34620.27</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>11906</v>
+        <v>2967</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>123698.6</v>
+        <v>30825.9</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>22.28</v>
+        <v>3.13</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>0.0001599638765773488</v>
+        <v>9.007919018030242e-05</v>
       </c>
       <c r="K10" s="12" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>0</v>
@@ -954,25 +954,25 @@
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>36493</v>
+        <v>15163</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>149520.08</v>
+        <v>64138.66</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>13415</v>
+        <v>5521</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>247675.8</v>
+        <v>101932</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>7317.57</v>
+        <v>406.37</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>0.04662197246990389</v>
+        <v>0.006290991505626536</v>
       </c>
       <c r="K12" s="12" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="L12" s="12" t="n">
         <v>492</v>
@@ -1009,25 +1009,25 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>7530</v>
+        <v>6270</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>37602.6</v>
+        <v>33343.8</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>3227</v>
+        <v>2873</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>75436.3</v>
+        <v>67161</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>123.61</v>
+        <v>245.14</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>0.00327384594195874</v>
+        <v>0.007292683724984456</v>
       </c>
       <c r="K13" s="12" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="L13" s="12" t="n">
         <v>1636</v>
@@ -1064,22 +1064,22 @@
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>3897</v>
+        <v>3537</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>4703.04</v>
+        <v>4663.44</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>11656.3</v>
+        <v>11598.6</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>6.29</v>
+        <v>24.29</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>0.001331767792163831</v>
+        <v>0.005163286133435387</v>
       </c>
       <c r="K14" s="12" t="n">
         <v>11</v>
@@ -1284,22 +1284,22 @@
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>1754</v>
+        <v>1214</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>19129.99</v>
+        <v>13465.39</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>1754</v>
+        <v>1214</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>129554.1</v>
+        <v>89668.60000000001</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>1389.02</v>
+        <v>735.62</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>0.06768499839195392</v>
+        <v>0.05179022515101592</v>
       </c>
       <c r="K18" s="12" t="n">
         <v>21</v>
@@ -1398,25 +1398,25 @@
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>143208</v>
+        <v>63105</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>453959.596</v>
+        <v>254286.406</v>
       </c>
       <c r="G20" s="22" t="n">
-        <v>37682</v>
+        <v>19953</v>
       </c>
       <c r="H20" s="24" t="n">
-        <v>792221.3999999999</v>
+        <v>505386.4299999999</v>
       </c>
       <c r="I20" s="23" t="n">
-        <v>11579.329</v>
+        <v>4135.089</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.02626416430434264</v>
+        <v>0.01771294593576957</v>
       </c>
       <c r="K20" s="26" t="n">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="L20" s="26" t="n">
         <v>5629</v>

</xml_diff>

<commit_message>
data(km19): sinh lại bộ file cắt thép sau khi đọc đủ Mố M1/M2, gờ lan can, liên tục nhiệt
- Nguồn: BBS đã sửa (thêm H1 R25/H2 R8 tròn trơn CB240-T, B1, U4, T1, T2 của mố; gờ lan can đủ 19 đốt;
  liên tục nhiệt L1/L2/L3/S4 × 2 vị trí). 0 lỗi đọc, 0 thanh chưa lập kế hoạch.
- 20.311 cây 11,7 m (bản trước 19.953), đề-xê chung 1,79%; Ø16 FEASIBLE (60 s/Ø), các Ø khác OPTIMAL.
  Thép tròn trơn được cắt nhóm riêng theo mác (CB240-T).
- Vẫn gồm W6, W7, W9 của Mố M2 (bản vẽ ghi 0 kg nhưng có dài và số lượng) — chờ chủ dự án quyết định.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/00_BANG_TONG_HOP_CAT_THEP_THEO_PHI.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/00_BANG_TONG_HOP_CAT_THEP_THEO_PHI.xlsx
@@ -734,25 +734,25 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>81</v>
+        <v>292</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>60.59</v>
+        <v>253.86</v>
       </c>
       <c r="G8" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>0.008492618492618493</v>
+      </c>
+      <c r="K8" s="12" t="n">
         <v>6</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="I8" s="9" t="n">
-        <v>9.23</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>0.1315242165242165</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>4</v>
       </c>
       <c r="L8" s="12" t="n">
         <v>0</v>
@@ -789,25 +789,25 @@
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>7419</v>
+        <v>7939</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>19352.59</v>
+        <v>19518.99</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>1663</v>
+        <v>1672</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>12005</v>
+        <v>12070</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>68.81</v>
+        <v>5.16</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.003536601035097728</v>
+        <v>0.0002636179609863821</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L9" s="12" t="n">
         <v>1384</v>
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>21068</v>
+        <v>22312</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>34620.27</v>
+        <v>35138.1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>2967</v>
+        <v>3012</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>30825.9</v>
+        <v>31293.5</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>3.13</v>
+        <v>5.8</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>9.007919018030242e-05</v>
+        <v>0.0001646689594896766</v>
       </c>
       <c r="K10" s="12" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>0</v>
@@ -899,25 +899,25 @@
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>3856</v>
+        <v>3925</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>28699.85</v>
+        <v>28740.21</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>2463</v>
+        <v>2464</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>34811.1</v>
+        <v>34825.2</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>102.73</v>
+        <v>73.72</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.003564758424685343</v>
+        <v>0.002557199744699745</v>
       </c>
       <c r="K11" s="12" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L11" s="12" t="n">
         <v>1512</v>
@@ -954,25 +954,25 @@
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>15163</v>
+        <v>15282</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>64138.66</v>
+        <v>64291.88</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>5521</v>
+        <v>5529</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>101932</v>
+        <v>102079.7</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>406.37</v>
+        <v>346.19</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>0.006290991505626536</v>
+        <v>0.005351657847588395</v>
       </c>
       <c r="K12" s="12" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L12" s="12" t="n">
         <v>492</v>
@@ -1009,28 +1009,28 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>6270</v>
+        <v>6594</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>33343.8</v>
+        <v>35215.98</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>2873</v>
+        <v>3035</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>67161</v>
+        <v>70948</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>245.14</v>
+        <v>267.01</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>0.007292683724984456</v>
+        <v>0.007519311733479773</v>
       </c>
       <c r="K13" s="12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>1636</v>
+        <v>1744</v>
       </c>
       <c r="M13" s="8" t="n">
         <v>0</v>
@@ -1174,25 +1174,25 @@
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>2808</v>
+        <v>3190</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>25549.61</v>
+        <v>26915.95</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>2302</v>
+        <v>2419</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>103774.4</v>
+        <v>109048.8</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>1381.14</v>
+        <v>1382.37</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>0.05127974930755122</v>
+        <v>0.04884313289025979</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L16" s="12" t="n">
         <v>24</v>
@@ -1398,28 +1398,28 @@
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>63105</v>
+        <v>65974</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>254286.406</v>
+        <v>258596.013</v>
       </c>
       <c r="G20" s="22" t="n">
-        <v>19953</v>
+        <v>20311</v>
       </c>
       <c r="H20" s="24" t="n">
-        <v>505386.4299999999</v>
+        <v>515216.1</v>
       </c>
       <c r="I20" s="23" t="n">
-        <v>4135.089</v>
+        <v>4000.987</v>
       </c>
       <c r="J20" s="25" t="n">
-        <v>0.01771294593576957</v>
+        <v>0.01683642857834183</v>
       </c>
       <c r="K20" s="26" t="n">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="L20" s="26" t="n">
-        <v>5629</v>
+        <v>5737</v>
       </c>
       <c r="M20" s="22" t="n">
         <v>0</v>

</xml_diff>